<commit_message>
Add ED per-SPU yield ladder metrics and January downgrade trigger to checkpoints
Co-authored-by: devlee <devlee@outlook.com>
</commit_message>
<xml_diff>
--- a/missacc_2027_growth_analysis/missacc_launch_plan_202608_202703.xlsx
+++ b/missacc_2027_growth_analysis/missacc_launch_plan_202608_202703.xlsx
@@ -1242,7 +1242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1386,6 +1386,57 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>ED单款产出阶梯①</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>0-6月新款单SPU月收入应≥$400；未达则收紧选款门槛，空坑位按条件规则让给BD（宁缺毋滥，坑位使用率不考核）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ED单款产出阶梯②/触发条款</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>应≥$450；未达则下调ED目标至+45%(v50)/+55%(v60)，缺口转MOB/BM超额空间，2-3月坑位减15-20/月转BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ED单款产出阶梯③</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>目标≥$500（参考自家3-6月队列已实测$523）；同步考核老款动销率18.9%→23-25%（每+1pp≈+$9.5K/月）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>